<commit_message>
Add the 3 new Hopfenstrasse units missing from Property Details
These units (2nd floor Left, ground floor Left, 1st floor Right at
Hopfenstrasse 15) only existed in the Apartments and Availability
sheet, not yet in Property Details. Generated Property IDs following
the sheet's existing convention (matches sibling units HO15-4L,
HO15-2R, HO15-3R at the same address), and filled Property Name,
Type, Object Number, Own/Sublet, size, room type, and status from the
apartments sheet. Fields with no source data stay blank, same as the
rest of the sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Property_Details_V4-RS-04.04.2026-v2.xlsx
+++ b/Property_Details_V4-RS-04.04.2026-v2.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB145"/>
+  <dimension ref="A1:AB148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14431,6 +14431,292 @@
       <c r="AB145" t="inlineStr">
         <is>
           <t>31st Oct '2025 | washing area common, dishwasher ,no balcony | Will be surrendered: 31st Oct '2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>HO15-2L-3.5-APA-SUB-8045-ZH-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>APARTMENT</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="n">
+        <v>10</v>
+      </c>
+      <c r="F146" t="n">
+        <v>1021</v>
+      </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>SUB</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Hopfenstrasse</t>
+        </is>
+      </c>
+      <c r="K146" t="n">
+        <v>15</v>
+      </c>
+      <c r="L146" t="n">
+        <v>8045</v>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr"/>
+      <c r="Q146" t="n">
+        <v>2</v>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="S146" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="T146" t="n">
+        <v>80</v>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="V146" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W146" t="inlineStr"/>
+      <c r="X146" t="inlineStr"/>
+      <c r="Y146" t="inlineStr"/>
+      <c r="Z146" t="inlineStr"/>
+      <c r="AA146" t="inlineStr"/>
+      <c r="AB146" t="inlineStr">
+        <is>
+          <t>will be rent from 1st april bt rent srt date 16th may 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>HO15-GL-3.5-APA-SUB-8045-ZH-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>APARTMENT</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="n">
+        <v>6</v>
+      </c>
+      <c r="F147" t="n">
+        <v>1001</v>
+      </c>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>SUB</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Hopfenstrasse</t>
+        </is>
+      </c>
+      <c r="K147" t="n">
+        <v>15</v>
+      </c>
+      <c r="L147" t="n">
+        <v>8045</v>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr"/>
+      <c r="Q147" t="n">
+        <v>0</v>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="S147" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="T147" t="n">
+        <v>80</v>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="V147" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W147" t="inlineStr"/>
+      <c r="X147" t="inlineStr"/>
+      <c r="Y147" t="inlineStr"/>
+      <c r="Z147" t="inlineStr"/>
+      <c r="AA147" t="inlineStr"/>
+      <c r="AB147" t="inlineStr">
+        <is>
+          <t>will be rent from 1st june bt rent srt date 16th july 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>HO15-1R-3.5-APA-SUB-8045-ZH-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>APARTMENT</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="n">
+        <v>1012</v>
+      </c>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>SUB</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Hopfenstrasse</t>
+        </is>
+      </c>
+      <c r="K148" t="n">
+        <v>15</v>
+      </c>
+      <c r="L148" t="n">
+        <v>8045</v>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr"/>
+      <c r="Q148" t="n">
+        <v>1</v>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="S148" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="T148" t="n">
+        <v>80</v>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="V148" t="inlineStr">
+        <is>
+          <t>NEW APARTMENT</t>
+        </is>
+      </c>
+      <c r="W148" t="inlineStr"/>
+      <c r="X148" t="inlineStr"/>
+      <c r="Y148" t="inlineStr"/>
+      <c r="Z148" t="inlineStr"/>
+      <c r="AA148" t="inlineStr"/>
+      <c r="AB148" t="inlineStr">
+        <is>
+          <t>will be rent from 1st oct 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 14 parking properties to Property Details
Imports parking_properties.csv (skipping the "142 PARKINGS" section
header row, which isn't a real record) into the Property Master sheet
as PARKING-type entries. For each spot: generated a Property ID
following the sheet's street-prefix + pincode + city-code + canton
convention (reusing the exact city codes already established for
Bonstatten/Glattbrugg/Embrach/Wallisellen/Zurich/Birmensdorf), filled
Object Number (from List Order), Parking/Garage Nr (the spot number),
address fields, and mapped Active/Inactive status to Occupied/Vacant.
Room type descriptions carried over into Remarks.

Also synced this into the live MongoDB property details data
collection so the dashboard reflects it immediately.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Property_Details_V4-RS-04.04.2026-v2.xlsx
+++ b/Property_Details_V4-RS-04.04.2026-v2.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB148"/>
+  <dimension ref="A1:AB162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14717,6 +14717,1154 @@
       <c r="AB148" t="inlineStr">
         <is>
           <t>will be rent from 1st oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>DO24-P14-PAR-8906-BO-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="n">
+        <v>143</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Dorfstrasse</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="L149" t="n">
+        <v>8906</v>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>Bonstatten</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr"/>
+      <c r="Q149" t="inlineStr"/>
+      <c r="R149" t="inlineStr"/>
+      <c r="S149" t="inlineStr"/>
+      <c r="T149" t="inlineStr"/>
+      <c r="U149" t="inlineStr"/>
+      <c r="V149" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W149" t="inlineStr"/>
+      <c r="X149" t="inlineStr"/>
+      <c r="Y149" t="inlineStr"/>
+      <c r="Z149" t="inlineStr"/>
+      <c r="AA149" t="inlineStr"/>
+      <c r="AB149" t="inlineStr">
+        <is>
+          <t>Covered/Underground parking. Parking NO(Covered/underground) -14 Dorfstrasse 24, 8906, Bonstatten</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>LA5-P4-PAR-8152-GB-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="n">
+        <v>144</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Lattenwiesenstrasse</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="L150" t="n">
+        <v>8152</v>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>Glattbrugg</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr"/>
+      <c r="Q150" t="inlineStr"/>
+      <c r="R150" t="inlineStr"/>
+      <c r="S150" t="inlineStr"/>
+      <c r="T150" t="inlineStr"/>
+      <c r="U150" t="inlineStr"/>
+      <c r="V150" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W150" t="inlineStr"/>
+      <c r="X150" t="inlineStr"/>
+      <c r="Y150" t="inlineStr"/>
+      <c r="Z150" t="inlineStr"/>
+      <c r="AA150" t="inlineStr"/>
+      <c r="AB150" t="inlineStr">
+        <is>
+          <t>Open parking. Open NO- 4, Lattenwiesenstarsse 5, 8152 Glattbrugg</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>JA4-P3-PAR-8424-EM-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="n">
+        <v>145</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Jakob Bosshart-Strasse</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="L151" t="n">
+        <v>8424</v>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>Embrach</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr"/>
+      <c r="Q151" t="inlineStr"/>
+      <c r="R151" t="inlineStr"/>
+      <c r="S151" t="inlineStr"/>
+      <c r="T151" t="inlineStr"/>
+      <c r="U151" t="inlineStr"/>
+      <c r="V151" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W151" t="inlineStr"/>
+      <c r="X151" t="inlineStr"/>
+      <c r="Y151" t="inlineStr"/>
+      <c r="Z151" t="inlineStr"/>
+      <c r="AA151" t="inlineStr"/>
+      <c r="AB151" t="inlineStr">
+        <is>
+          <t>Covered/Underground (PG) parking. PG - Parking No - 3 - Jakob Bosshart-Strasse 4, 8424 Embrach – 4.5 Room Apartment</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>NE16-P8-PAR-8304-WS-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="n">
+        <v>146</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Neugutstrasse</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="L152" t="n">
+        <v>8304</v>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>Wallisellen</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr"/>
+      <c r="Q152" t="inlineStr"/>
+      <c r="R152" t="inlineStr"/>
+      <c r="S152" t="inlineStr"/>
+      <c r="T152" t="inlineStr"/>
+      <c r="U152" t="inlineStr"/>
+      <c r="V152" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W152" t="inlineStr"/>
+      <c r="X152" t="inlineStr"/>
+      <c r="Y152" t="inlineStr"/>
+      <c r="Z152" t="inlineStr"/>
+      <c r="AA152" t="inlineStr"/>
+      <c r="AB152" t="inlineStr">
+        <is>
+          <t>Open parking. Open No. - 8,Neugutstrasse 16 8304 Wallisellen</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>SE66-P3-PAR-8052-ZH-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="n">
+        <v>148</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Seebacherstrasse</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="L153" t="n">
+        <v>8052</v>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr"/>
+      <c r="Q153" t="inlineStr"/>
+      <c r="R153" t="inlineStr"/>
+      <c r="S153" t="inlineStr"/>
+      <c r="T153" t="inlineStr"/>
+      <c r="U153" t="inlineStr"/>
+      <c r="V153" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W153" t="inlineStr"/>
+      <c r="X153" t="inlineStr"/>
+      <c r="Y153" t="inlineStr"/>
+      <c r="Z153" t="inlineStr"/>
+      <c r="AA153" t="inlineStr"/>
+      <c r="AB153" t="inlineStr">
+        <is>
+          <t>Open parking. Open No. - 3, Seebacherstrasse 66, 8052, Zurich - 2.5 Zi</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>ST40A-P100-PAR-8903-BD-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="n">
+        <v>149</v>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Stöckenstrasse</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>40a</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>8903</v>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>Birmensdorf</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr"/>
+      <c r="Q154" t="inlineStr"/>
+      <c r="R154" t="inlineStr"/>
+      <c r="S154" t="inlineStr"/>
+      <c r="T154" t="inlineStr"/>
+      <c r="U154" t="inlineStr"/>
+      <c r="V154" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W154" t="inlineStr"/>
+      <c r="X154" t="inlineStr"/>
+      <c r="Y154" t="inlineStr"/>
+      <c r="Z154" t="inlineStr"/>
+      <c r="AA154" t="inlineStr"/>
+      <c r="AB154" t="inlineStr">
+        <is>
+          <t>Covered/Underground parking. Covered / Underground Parking Nr – 100;Stöckenstrasse 40a, 8903, Birmensdorf</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>TA47-P9-PAR-8152-GB-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr"/>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="n">
+        <v>150</v>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Talackerstrasse</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L155" t="n">
+        <v>8152</v>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>Glattbrugg</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr"/>
+      <c r="Q155" t="inlineStr"/>
+      <c r="R155" t="inlineStr"/>
+      <c r="S155" t="inlineStr"/>
+      <c r="T155" t="inlineStr"/>
+      <c r="U155" t="inlineStr"/>
+      <c r="V155" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W155" t="inlineStr"/>
+      <c r="X155" t="inlineStr"/>
+      <c r="Y155" t="inlineStr"/>
+      <c r="Z155" t="inlineStr"/>
+      <c r="AA155" t="inlineStr"/>
+      <c r="AB155" t="inlineStr">
+        <is>
+          <t>Open parking. Open No.– 9; Talackerstrasse 47, 8152, Glattbrugg - 3.5 Zi</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>TA47-P7-PAR-8152-GB-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr"/>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="n">
+        <v>151</v>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Talackerstrasse</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L156" t="n">
+        <v>8152</v>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>Glattbrugg</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr"/>
+      <c r="Q156" t="inlineStr"/>
+      <c r="R156" t="inlineStr"/>
+      <c r="S156" t="inlineStr"/>
+      <c r="T156" t="inlineStr"/>
+      <c r="U156" t="inlineStr"/>
+      <c r="V156" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W156" t="inlineStr"/>
+      <c r="X156" t="inlineStr"/>
+      <c r="Y156" t="inlineStr"/>
+      <c r="Z156" t="inlineStr"/>
+      <c r="AA156" t="inlineStr"/>
+      <c r="AB156" t="inlineStr">
+        <is>
+          <t>Open parking. Open No. – 7 ; Talackerstrasse 47, 8152, Glattbrugg - 4.5 Zi</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>WA156-P176-PAR-8152-GB-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="n">
+        <v>152</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Wallisellerstrasse</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="L157" t="n">
+        <v>8152</v>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>Glattbrugg</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr"/>
+      <c r="Q157" t="inlineStr"/>
+      <c r="R157" t="inlineStr"/>
+      <c r="S157" t="inlineStr"/>
+      <c r="T157" t="inlineStr"/>
+      <c r="U157" t="inlineStr"/>
+      <c r="V157" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W157" t="inlineStr"/>
+      <c r="X157" t="inlineStr"/>
+      <c r="Y157" t="inlineStr"/>
+      <c r="Z157" t="inlineStr"/>
+      <c r="AA157" t="inlineStr"/>
+      <c r="AB157" t="inlineStr">
+        <is>
+          <t>Covered/Underground parking. Covered / Underground NO. – 176 ; Wallisellerstrasse 156, 8152, Glattbrugg - 3.5 Zi</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>AL18-P8-PAR-8304-WS-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr"/>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="n">
+        <v>153</v>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr"/>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Allmendstrasse</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="L158" t="n">
+        <v>8304</v>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>Wallisellen</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr"/>
+      <c r="Q158" t="inlineStr"/>
+      <c r="R158" t="inlineStr"/>
+      <c r="S158" t="inlineStr"/>
+      <c r="T158" t="inlineStr"/>
+      <c r="U158" t="inlineStr"/>
+      <c r="V158" t="inlineStr">
+        <is>
+          <t>VACANT</t>
+        </is>
+      </c>
+      <c r="W158" t="inlineStr"/>
+      <c r="X158" t="inlineStr"/>
+      <c r="Y158" t="inlineStr"/>
+      <c r="Z158" t="inlineStr"/>
+      <c r="AA158" t="inlineStr"/>
+      <c r="AB158" t="inlineStr">
+        <is>
+          <t>Open parking. Open NO. – 8; Allmendstrasse 18, 8304 Wallisellen – 3.5 Zi</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>WA156-P24-PAR-8152-GB-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="n">
+        <v>154</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr"/>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Wallisellerstrasse</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="L159" t="n">
+        <v>8152</v>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>Glattbrugg</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr"/>
+      <c r="Q159" t="inlineStr"/>
+      <c r="R159" t="inlineStr"/>
+      <c r="S159" t="inlineStr"/>
+      <c r="T159" t="inlineStr"/>
+      <c r="U159" t="inlineStr"/>
+      <c r="V159" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W159" t="inlineStr"/>
+      <c r="X159" t="inlineStr"/>
+      <c r="Y159" t="inlineStr"/>
+      <c r="Z159" t="inlineStr"/>
+      <c r="AA159" t="inlineStr"/>
+      <c r="AB159" t="inlineStr">
+        <is>
+          <t>Open parking. Open No. - 24; Wallisellerstrasse 156, 8152, Glattbrugg - 2.5 Zi</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>ME10-P73-PAR-8304-WS-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="n">
+        <v>159</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Melchrütistrasse</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L160" t="n">
+        <v>8304</v>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>Wallisellen</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr"/>
+      <c r="Q160" t="inlineStr"/>
+      <c r="R160" t="inlineStr"/>
+      <c r="S160" t="inlineStr"/>
+      <c r="T160" t="inlineStr"/>
+      <c r="U160" t="inlineStr"/>
+      <c r="V160" t="inlineStr">
+        <is>
+          <t>VACANT</t>
+        </is>
+      </c>
+      <c r="W160" t="inlineStr"/>
+      <c r="X160" t="inlineStr"/>
+      <c r="Y160" t="inlineStr"/>
+      <c r="Z160" t="inlineStr"/>
+      <c r="AA160" t="inlineStr"/>
+      <c r="AB160" t="inlineStr">
+        <is>
+          <t>Parking Lot parking. Parking Lot Nr 73 - Melchrütistrasse 10, 8304 Wallisellen</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>ME10-P24-PAR-8304-WS-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="inlineStr"/>
+      <c r="F161" t="n">
+        <v>171</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Melchrütistrasse</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L161" t="n">
+        <v>8304</v>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>Wallisellen</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr"/>
+      <c r="Q161" t="inlineStr"/>
+      <c r="R161" t="inlineStr"/>
+      <c r="S161" t="inlineStr"/>
+      <c r="T161" t="inlineStr"/>
+      <c r="U161" t="inlineStr"/>
+      <c r="V161" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W161" t="inlineStr"/>
+      <c r="X161" t="inlineStr"/>
+      <c r="Y161" t="inlineStr"/>
+      <c r="Z161" t="inlineStr"/>
+      <c r="AA161" t="inlineStr"/>
+      <c r="AB161" t="inlineStr">
+        <is>
+          <t>Parking parking. Parking Nr 24 - Melchrütistrasse 10, 8304 Wallisellen</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>ME8-P89-PAR-8304-WS-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="n">
+        <v>172</v>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Melchrütistrasse</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L162" t="n">
+        <v>8304</v>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>Wallisellen</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr"/>
+      <c r="Q162" t="inlineStr"/>
+      <c r="R162" t="inlineStr"/>
+      <c r="S162" t="inlineStr"/>
+      <c r="T162" t="inlineStr"/>
+      <c r="U162" t="inlineStr"/>
+      <c r="V162" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W162" t="inlineStr"/>
+      <c r="X162" t="inlineStr"/>
+      <c r="Y162" t="inlineStr"/>
+      <c r="Z162" t="inlineStr"/>
+      <c r="AA162" t="inlineStr"/>
+      <c r="AB162" t="inlineStr">
+        <is>
+          <t>Parking parking. Parking Nr 89 - Melchrütistrasse 8, 8304 Wallisellen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 3 new parking/garage units found in Parking_Units_Report.xls
Compared the report against the existing 14 parking entries and added
only the ones missing: Seebacherstrasse 64 spot 16, Albisstrasse 55
Garage 32 (first GARAGE-type entry), and Auf der Fuhren 435 Open Plot
4665-2. Guest/tenant names from the report are recorded in Remarks.
Existing parking entries were left untouched, including one status
discrepancy noted separately (Jakob Bosshart-Strasse 4 spot 3 shows
Occupied in Property Details but Vacant in this new report).

Synced into MongoDB so the dashboard reflects it immediately.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Property_Details_V4-RS-04.04.2026-v2.xlsx
+++ b/Property_Details_V4-RS-04.04.2026-v2.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB162"/>
+  <dimension ref="A1:AB165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14741,10 +14741,8 @@
       <c r="F149" t="n">
         <v>143</v>
       </c>
-      <c r="G149" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="G149" t="n">
+        <v>14</v>
       </c>
       <c r="H149" t="inlineStr">
         <is>
@@ -14823,10 +14821,8 @@
       <c r="F150" t="n">
         <v>144</v>
       </c>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="G150" t="n">
+        <v>4</v>
       </c>
       <c r="H150" t="inlineStr">
         <is>
@@ -14905,10 +14901,8 @@
       <c r="F151" t="n">
         <v>145</v>
       </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G151" t="n">
+        <v>3</v>
       </c>
       <c r="H151" t="inlineStr">
         <is>
@@ -14987,10 +14981,8 @@
       <c r="F152" t="n">
         <v>146</v>
       </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="G152" t="n">
+        <v>8</v>
       </c>
       <c r="H152" t="inlineStr">
         <is>
@@ -15069,10 +15061,8 @@
       <c r="F153" t="n">
         <v>148</v>
       </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G153" t="n">
+        <v>3</v>
       </c>
       <c r="H153" t="inlineStr">
         <is>
@@ -15151,10 +15141,8 @@
       <c r="F154" t="n">
         <v>149</v>
       </c>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="G154" t="n">
+        <v>100</v>
       </c>
       <c r="H154" t="inlineStr">
         <is>
@@ -15233,10 +15221,8 @@
       <c r="F155" t="n">
         <v>150</v>
       </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
+      <c r="G155" t="n">
+        <v>9</v>
       </c>
       <c r="H155" t="inlineStr">
         <is>
@@ -15315,10 +15301,8 @@
       <c r="F156" t="n">
         <v>151</v>
       </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="G156" t="n">
+        <v>7</v>
       </c>
       <c r="H156" t="inlineStr">
         <is>
@@ -15397,10 +15381,8 @@
       <c r="F157" t="n">
         <v>152</v>
       </c>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>176</t>
-        </is>
+      <c r="G157" t="n">
+        <v>176</v>
       </c>
       <c r="H157" t="inlineStr">
         <is>
@@ -15479,10 +15461,8 @@
       <c r="F158" t="n">
         <v>153</v>
       </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="G158" t="n">
+        <v>8</v>
       </c>
       <c r="H158" t="inlineStr">
         <is>
@@ -15561,10 +15541,8 @@
       <c r="F159" t="n">
         <v>154</v>
       </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="G159" t="n">
+        <v>24</v>
       </c>
       <c r="H159" t="inlineStr">
         <is>
@@ -15643,10 +15621,8 @@
       <c r="F160" t="n">
         <v>159</v>
       </c>
-      <c r="G160" t="inlineStr">
-        <is>
-          <t>73</t>
-        </is>
+      <c r="G160" t="n">
+        <v>73</v>
       </c>
       <c r="H160" t="inlineStr">
         <is>
@@ -15725,10 +15701,8 @@
       <c r="F161" t="n">
         <v>171</v>
       </c>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="G161" t="n">
+        <v>24</v>
       </c>
       <c r="H161" t="inlineStr">
         <is>
@@ -15807,10 +15781,8 @@
       <c r="F162" t="n">
         <v>172</v>
       </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
+      <c r="G162" t="n">
+        <v>89</v>
       </c>
       <c r="H162" t="inlineStr">
         <is>
@@ -15865,6 +15837,242 @@
       <c r="AB162" t="inlineStr">
         <is>
           <t>Parking parking. Parking Nr 89 - Melchrütistrasse 8, 8304 Wallisellen</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>SE64-P16-PAR-8052-ZH-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="n">
+        <v>16</v>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Seebacherstrasse</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="L163" t="n">
+        <v>8052</v>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr"/>
+      <c r="Q163" t="inlineStr"/>
+      <c r="R163" t="inlineStr"/>
+      <c r="S163" t="inlineStr"/>
+      <c r="T163" t="inlineStr"/>
+      <c r="U163" t="inlineStr"/>
+      <c r="V163" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W163" t="inlineStr"/>
+      <c r="X163" t="inlineStr"/>
+      <c r="Y163" t="inlineStr"/>
+      <c r="Z163" t="inlineStr"/>
+      <c r="AA163" t="inlineStr"/>
+      <c r="AB163" t="inlineStr">
+        <is>
+          <t>Open parking No.16. Guest/Tenant: Mr. Kawa Osman</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>AL55-G32-GAR-8134-AW-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>GARAGE</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="n">
+        <v>32</v>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Albisstrasse</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="L164" t="n">
+        <v>8134</v>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>Adliswil</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr"/>
+      <c r="Q164" t="inlineStr"/>
+      <c r="R164" t="inlineStr"/>
+      <c r="S164" t="inlineStr"/>
+      <c r="T164" t="inlineStr"/>
+      <c r="U164" t="inlineStr"/>
+      <c r="V164" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W164" t="inlineStr"/>
+      <c r="X164" t="inlineStr"/>
+      <c r="Y164" t="inlineStr"/>
+      <c r="Z164" t="inlineStr"/>
+      <c r="AA164" t="inlineStr"/>
+      <c r="AB164" t="inlineStr">
+        <is>
+          <t>Garage No.32. Guest/Tenant: Bukurim Limani</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>AU435-P4665_2-PAR-3822-LB-BE-CH</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>PARKING</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>4665-2</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Auf der Fuhren</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>435</t>
+        </is>
+      </c>
+      <c r="L165" t="n">
+        <v>3822</v>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>Lauterbrunnen</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr"/>
+      <c r="Q165" t="inlineStr"/>
+      <c r="R165" t="inlineStr"/>
+      <c r="S165" t="inlineStr"/>
+      <c r="T165" t="inlineStr"/>
+      <c r="U165" t="inlineStr"/>
+      <c r="V165" t="inlineStr">
+        <is>
+          <t>OCCUPIED</t>
+        </is>
+      </c>
+      <c r="W165" t="inlineStr"/>
+      <c r="X165" t="inlineStr"/>
+      <c r="Y165" t="inlineStr"/>
+      <c r="Z165" t="inlineStr"/>
+      <c r="AA165" t="inlineStr"/>
+      <c r="AB165" t="inlineStr">
+        <is>
+          <t>Open Plot No.4665-2. Guest/Tenant: Mr. Anton Graf Kammer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split parking Property ID type code by parking sub-type
Replaces the generic PAR/GAR type segment in parking Property IDs with
a code specific to the sub-type, keeping every other ID segment
unchanged:
  Open parking            -> OP
  Covered/Underground      -> BP (basement)
  Garage                   -> GP

All 17 parking/garage entries updated (14 existing + 3 added from the
Parking_Units_Report.xls import). Synced into MongoDB.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Property_Details_V4-RS-04.04.2026-v2.xlsx
+++ b/Property_Details_V4-RS-04.04.2026-v2.xlsx
@@ -14723,7 +14723,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>DO24-P14-PAR-8906-BO-ZH-CH</t>
+          <t>DO24-P14-BP-8906-BO-ZH-CH</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -14803,7 +14803,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>LA5-P4-PAR-8152-GB-ZH-CH</t>
+          <t>LA5-P4-OP-8152-GB-ZH-CH</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -14883,7 +14883,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>JA4-P3-PAR-8424-EM-ZH-CH</t>
+          <t>JA4-P3-BP-8424-EM-ZH-CH</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -14963,7 +14963,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>NE16-P8-PAR-8304-WS-ZH-CH</t>
+          <t>NE16-P8-OP-8304-WS-ZH-CH</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -15043,7 +15043,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SE66-P3-PAR-8052-ZH-ZH-CH</t>
+          <t>SE66-P3-OP-8052-ZH-ZH-CH</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -15123,7 +15123,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>ST40A-P100-PAR-8903-BD-ZH-CH</t>
+          <t>ST40A-P100-BP-8903-BD-ZH-CH</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -15203,7 +15203,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>TA47-P9-PAR-8152-GB-ZH-CH</t>
+          <t>TA47-P9-OP-8152-GB-ZH-CH</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -15283,7 +15283,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>TA47-P7-PAR-8152-GB-ZH-CH</t>
+          <t>TA47-P7-OP-8152-GB-ZH-CH</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -15363,7 +15363,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>WA156-P176-PAR-8152-GB-ZH-CH</t>
+          <t>WA156-P176-BP-8152-GB-ZH-CH</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -15443,7 +15443,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>AL18-P8-PAR-8304-WS-ZH-CH</t>
+          <t>AL18-P8-OP-8304-WS-ZH-CH</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -15523,7 +15523,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>WA156-P24-PAR-8152-GB-ZH-CH</t>
+          <t>WA156-P24-OP-8152-GB-ZH-CH</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -15603,7 +15603,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ME10-P73-PAR-8304-WS-ZH-CH</t>
+          <t>ME10-P73-OP-8304-WS-ZH-CH</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -15683,7 +15683,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ME10-P24-PAR-8304-WS-ZH-CH</t>
+          <t>ME10-P24-OP-8304-WS-ZH-CH</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -15763,7 +15763,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>ME8-P89-PAR-8304-WS-ZH-CH</t>
+          <t>ME8-P89-OP-8304-WS-ZH-CH</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -15843,7 +15843,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SE64-P16-PAR-8052-ZH-ZH-CH</t>
+          <t>SE64-P16-OP-8052-ZH-ZH-CH</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -15921,7 +15921,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>AL55-G32-GAR-8134-AW-ZH-CH</t>
+          <t>AL55-G32-GP-8134-AW-ZH-CH</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -15999,7 +15999,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>AU435-P4665_2-PAR-3822-LB-BE-CH</t>
+          <t>AU435-P4665_2-OP-3822-LB-BE-CH</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">

</xml_diff>

<commit_message>
Add Neugutstrasse 16, Wallisellen as an OFFICE property
This is Sinha's GmbH's own registered office address (also seen as
the letterhead on the Booking List export). Added as PROPERTY ID
NE16-X-X-OFF-OWN-8304-WS-ZH-CH, Own/Sublet=OWN since it's the
company's own office, floor/position unknown. Synced into MongoDB.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Property_Details_V4-RS-04.04.2026-v2.xlsx
+++ b/Property_Details_V4-RS-04.04.2026-v2.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB165"/>
+  <dimension ref="A1:AB166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16073,6 +16073,82 @@
       <c r="AB165" t="inlineStr">
         <is>
           <t>Open Plot No.4665-2. Guest/Tenant: Mr. Anton Graf Kammer</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>NE16-X-X-OFF-OWN-8304-WS-ZH-CH</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>SINHAS</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>OFFICE</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>NON OTA</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>OWN</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Neugutstrasse</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="L166" t="n">
+        <v>8304</v>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>Wallisellen</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>ZH</t>
+        </is>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr"/>
+      <c r="Q166" t="inlineStr"/>
+      <c r="R166" t="inlineStr"/>
+      <c r="S166" t="inlineStr"/>
+      <c r="T166" t="inlineStr"/>
+      <c r="U166" t="inlineStr"/>
+      <c r="V166" t="inlineStr"/>
+      <c r="W166" t="inlineStr"/>
+      <c r="X166" t="inlineStr"/>
+      <c r="Y166" t="inlineStr"/>
+      <c r="Z166" t="inlineStr"/>
+      <c r="AA166" t="inlineStr"/>
+      <c r="AB166" t="inlineStr">
+        <is>
+          <t>Sinha's GmbH registered office address</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Normalize Own/Sublet values to SUBLET in Property Details
The dropdown for this field offers OWN/SUBLET, but 125 records still
held the old abbreviated "SUB" value, which didn't match either option
and showed up as a stray extra choice in the admin panel dropdown.
Converted all of them to SUBLET in both MongoDB and the source Excel
file so the dropdown is clean.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Property_Details_V4-RS-04.04.2026-v2.xlsx
+++ b/Property_Details_V4-RS-04.04.2026-v2.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4854,7 +4854,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5228,7 +5228,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5422,7 +5422,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -5810,7 +5810,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -6484,7 +6484,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -6582,7 +6582,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -6680,7 +6680,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -6774,7 +6774,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -6868,7 +6868,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -6962,7 +6962,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -7154,7 +7154,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -7250,7 +7250,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -7344,7 +7344,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -7534,7 +7534,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -7734,7 +7734,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -7928,7 +7928,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -8128,7 +8128,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -8332,7 +8332,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -8434,7 +8434,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -8626,7 +8626,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -9118,7 +9118,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -9220,7 +9220,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -9318,7 +9318,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -9412,7 +9412,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -9608,7 +9608,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -9804,7 +9804,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -9900,7 +9900,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -10003,7 +10003,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -10099,7 +10099,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -10197,7 +10197,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -10293,7 +10293,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -10487,7 +10487,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -10583,7 +10583,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -10681,7 +10681,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -10775,7 +10775,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -10869,7 +10869,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -10967,7 +10967,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -11063,7 +11063,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -11157,7 +11157,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -11253,7 +11253,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -11347,7 +11347,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -11441,7 +11441,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -11539,7 +11539,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -11731,7 +11731,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -11829,7 +11829,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -11927,7 +11927,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -12225,7 +12225,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
@@ -12327,7 +12327,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -12429,7 +12429,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -12531,7 +12531,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -12725,7 +12725,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -12917,7 +12917,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -13015,7 +13015,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -13107,7 +13107,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -13295,7 +13295,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -13379,7 +13379,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -13745,7 +13745,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -13837,7 +13837,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -13929,7 +13929,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -14203,7 +14203,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
@@ -14293,7 +14293,7 @@
       <c r="H144" t="inlineStr"/>
       <c r="I144" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
@@ -14367,7 +14367,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
@@ -14465,7 +14465,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
@@ -14561,7 +14561,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
@@ -14655,7 +14655,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>SUB</t>
+          <t>SUBLET</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">

</xml_diff>